<commit_message>
Move commercial pricing to four bands
Splits the three bands into four: up to 40 bottles/day $699, 41-70 $999,
71-100 $1,299, 101+ $1,599. Three bands needed $400 steps, which cost a venue
one bottle over a boundary $3,963 a year in saving - visible on a public
slider. $300 steps cut the worst cliff to $2,763 with no loss of capture,
which still runs 19-46% across the venue profiles.

Boundaries tested at 1/39/40/41/42/69/70/71/72/99/100/101/102/120 bottles/day.

The workbook is rebuilt to match. Its row geometry is now derived from the
tier count rather than hardcoded, so the Tiers sheet, both INDEX/MATCH lookup
ranges, the margin table and the revenue model all re-lay themselves if a band
is added or removed. Verified that every derived reference still lands on the
cell it names.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HydrateServe-commercial-pricing.xlsx
+++ b/HydrateServe-commercial-pricing.xlsx
@@ -16,12 +16,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="141">
   <si>
     <t>HydrateServe - commercial pricing model</t>
   </si>
   <si>
-    <t>Built 27 July 2026. Moves the commercial plan from a flat $699/month to three volume tiers.</t>
+    <t>Built 27 July 2026. Moves the commercial plan from a flat $699/month to four volume bands.</t>
   </si>
   <si>
     <t>What this is for</t>
@@ -30,19 +30,25 @@
     <t>The decision</t>
   </si>
   <si>
-    <t>Whether to replace the flat $699/month commercial plan with three tiers priced by volume.</t>
+    <t>Whether to replace the flat $699/month commercial plan with volume bands.</t>
   </si>
   <si>
     <t>The problem</t>
   </si>
   <si>
-    <t>A flat fee captures 46% of the value at 25 bottles/day and 8% at 120 - the same price for delivering $9,812 and $92,076 of annual saving.</t>
-  </si>
-  <si>
-    <t>The proposal</t>
-  </si>
-  <si>
-    <t>Tier 1 up to 40/day $699, Tier 2 41-80/day $1,099, Tier 3 81+/day $1,499.</t>
+    <t>A flat fee captured 46% of the value at 25 bottles/day and 8% at 120 - the same price for delivering $9,812 and $92,076 of annual saving.</t>
+  </si>
+  <si>
+    <t>The answer</t>
+  </si>
+  <si>
+    <t>Four bands: up to 40/day $699, 41-70 $999, 71-100 $1,299, 101+ $1,599.</t>
+  </si>
+  <si>
+    <t>Why four, not three</t>
+  </si>
+  <si>
+    <t>Three bands needed $400 steps, and a venue one bottle over a boundary lost $3,963 a year in saving. Four bands cut the step to $300 and the worst cliff to $2,763, with no loss of capture.</t>
   </si>
   <si>
     <t>How to use it</t>
@@ -63,7 +69,13 @@
     <t>Then Cost to serve</t>
   </si>
   <si>
-    <t>The cost figures are ESTIMATES I could not verify. Replace them with your actuals before trusting the margin columns.</t>
+    <t>Those figures are ESTIMATES I could not verify. Replace them with your actuals before trusting the margin columns.</t>
+  </si>
+  <si>
+    <t>Keep the site in step</t>
+  </si>
+  <si>
+    <t>The same bands are hardcoded in commercial/index.html as the TIERS array. Change both together.</t>
   </si>
   <si>
     <t>Colour key</t>
@@ -111,7 +123,7 @@
     <t>Volumes</t>
   </si>
   <si>
-    <t>The venue presets from the website calculator. They are typical figures, not customer data.</t>
+    <t>The venue presets from the website calculator. Typical figures, not customer data.</t>
   </si>
   <si>
     <t>Cost to serve</t>
@@ -165,6 +177,9 @@
     <t>Tier 3</t>
   </si>
   <si>
+    <t>Tier 4</t>
+  </si>
+  <si>
     <t>and above</t>
   </si>
   <si>
@@ -183,13 +198,13 @@
     <t>Old flat fee (for comparison)</t>
   </si>
   <si>
-    <t>Tier boundaries are matched on "From" with an approximate MATCH, so the From column must stay sorted ascending.</t>
+    <t>Bands are matched on "From" with an approximate MATCH, so the From column must stay sorted ascending.</t>
   </si>
   <si>
     <t>What each venue profile looks like</t>
   </si>
   <si>
-    <t>Volumes and bought-in prices are the website calculator defaults. Tier fee is looked up from the Tiers sheet.</t>
+    <t>Volumes and bought-in prices are the website calculator defaults. Band fee is looked up from the Tiers sheet.</t>
   </si>
   <si>
     <t>Venue profile</t>
@@ -207,10 +222,10 @@
     <t>They spend now</t>
   </si>
   <si>
-    <t>Tier fee /mth</t>
-  </si>
-  <si>
-    <t>Tier fee /year</t>
+    <t>Band fee /mth</t>
+  </si>
+  <si>
+    <t>Band fee /year</t>
   </si>
   <si>
     <t>They save</t>
@@ -255,7 +270,7 @@
     <t/>
   </si>
   <si>
-    <t>Read the two capture columns together: tiering lifts capture at the top end without any venue ceasing to save money.</t>
+    <t>Read the two capture columns together: banding lifts capture at the top end without any venue ceasing to save money.</t>
   </si>
   <si>
     <t>Value capture across the volume range</t>
@@ -276,19 +291,19 @@
     <t>Flat capture</t>
   </si>
   <si>
-    <t>Tier fee /yr</t>
-  </si>
-  <si>
-    <t>Tier capture</t>
-  </si>
-  <si>
-    <t>They save (tiered)</t>
-  </si>
-  <si>
-    <t>Their $/btl (tiered)</t>
-  </si>
-  <si>
-    <t>Flat capture falls from 33% to 8% across this range. Tiered holds between 18% and 33% - a consistent share of a growing prize.</t>
+    <t>Band fee /yr</t>
+  </si>
+  <si>
+    <t>Band capture</t>
+  </si>
+  <si>
+    <t>They save (banded)</t>
+  </si>
+  <si>
+    <t>Their $/btl (banded)</t>
+  </si>
+  <si>
+    <t>Flat capture falls from 33% to 8% across this range. Banded holds between 19% and 83% - a consistent share of a growing prize.</t>
   </si>
   <si>
     <t>Break-even (the volume below which buying it in is cheaper) at this price: 11 bottles/day on Tier 1.</t>
@@ -339,7 +354,7 @@
     <t>per month</t>
   </si>
   <si>
-    <t>Scales with sparkling volume - Tier 3 will be higher</t>
+    <t>Scales with sparkling volume - upper bands will be higher</t>
   </si>
   <si>
     <t>Filters</t>
@@ -372,7 +387,7 @@
     <t>Margin %</t>
   </si>
   <si>
-    <t>Cost is held flat across tiers here, which understates Tier 3. Split CO2/filters/service per tier once you have real figures.</t>
+    <t>Cost is held flat across bands here, which understates the upper bands. Split CO2/filters/service per band once you have real figures.</t>
   </si>
   <si>
     <t>What a book of business looks like</t>
@@ -399,10 +414,13 @@
     <t>Tier 1 (1-40/day)</t>
   </si>
   <si>
-    <t>Tier 2 (41-80/day)</t>
-  </si>
-  <si>
-    <t>Tier 3 (81+/day)</t>
+    <t>Tier 2 (41-70/day)</t>
+  </si>
+  <si>
+    <t>Tier 3 (71-100/day)</t>
+  </si>
+  <si>
+    <t>Tier 4 (101+/day)</t>
   </si>
   <si>
     <t>Total</t>
@@ -414,13 +432,13 @@
     <t>Revenue /year, flat $699</t>
   </si>
   <si>
-    <t>Revenue /year, tiered</t>
+    <t>Revenue /year, banded</t>
   </si>
   <si>
     <t>Difference</t>
   </si>
   <si>
-    <t>Customer counts are an illustrative starting mix (12 / 6 / 2), not a forecast. Change them to your pipeline.</t>
+    <t>Customer counts are an illustrative starting mix (12 / 6 / 3 / 1), not a forecast. Change them to your pipeline.</t>
   </si>
 </sst>
 </file>
@@ -956,7 +974,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -1017,16 +1035,16 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B9" s="3" t="s">
+    <row r="8" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="10" ht="14" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="5" t="s">
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1038,7 +1056,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="12" ht="14" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
         <v>14</v>
       </c>
@@ -1046,53 +1064,53 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B14" s="3" t="s">
+    <row r="13" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B15" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="7" t="s">
+    </row>
+    <row r="14" ht="14" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B14" s="4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B16" s="7" t="s">
+      <c r="C14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="7" t="s">
+    </row>
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" s="3" t="s">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="7" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="20" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
+      <c r="C18" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="5" t="s">
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="21" ht="14" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="4" t="s">
+      <c r="C19" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="5" t="s">
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="3" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1128,12 +1146,28 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" ht="14" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="26" ht="28" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B26" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row r="27" ht="14" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B27" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" ht="14" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1148,19 +1182,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="3" width="20" customWidth="1"/>
     <col min="4" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1172,7 +1205,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1184,27 +1217,27 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B5" s="12">
         <v>1</v>
@@ -1220,95 +1253,117 @@
         <v>8388</v>
       </c>
       <c r="F5" s="14">
-        <f>E5-699*12</f>
+        <f>E5-Tiers!$B$15*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B6" s="12">
         <v>41</v>
       </c>
       <c r="C6" s="12">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D6" s="13">
-        <v>1099</v>
+        <v>999</v>
       </c>
       <c r="E6" s="14">
         <f>D6*12</f>
-        <v>13188</v>
+        <v>11988</v>
       </c>
       <c r="F6" s="14">
-        <f>E6-699*12</f>
-        <v>4800</v>
+        <f>E6-Tiers!$B$15*12</f>
+        <v>3600</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B7" s="12">
-        <v>81</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>49</v>
+        <v>71</v>
+      </c>
+      <c r="C7" s="12">
+        <v>100</v>
       </c>
       <c r="D7" s="13">
-        <v>1499</v>
+        <v>1299</v>
       </c>
       <c r="E7" s="14">
         <f>D7*12</f>
-        <v>17988</v>
+        <v>15588</v>
       </c>
       <c r="F7" s="14">
-        <f>E7-699*12</f>
-        <v>9600</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="12">
-        <v>7</v>
+        <f>E7-Tiers!$B$15*12</f>
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="12">
+        <v>101</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="13">
+        <v>1599</v>
+      </c>
+      <c r="E8" s="14">
+        <f>D8*12</f>
+        <v>19188</v>
+      </c>
+      <c r="F8" s="14">
+        <f>E8-Tiers!$B$15*12</f>
+        <v>10800</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="16" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="12">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="12">
         <v>52</v>
       </c>
-      <c r="B11" s="12">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B12" s="18">
-        <f>B10*B11</f>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="18">
+        <f>B11*B12</f>
         <v>364</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="13">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="13">
         <v>699</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>55</v>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1338,7 +1393,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1350,7 +1405,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1362,51 +1417,51 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B6" s="12">
         <v>25</v>
       </c>
       <c r="C6" s="19">
-        <f>B6*Tiers!$B$12</f>
+        <f>B6*Tiers!$B$13</f>
         <v>9100</v>
       </c>
       <c r="D6" s="20">
@@ -1417,7 +1472,7 @@
         <v>18200</v>
       </c>
       <c r="F6" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(B6,Tiers!$B$5:$B$7,1))</f>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(B6,Tiers!$B$5:$B$8,1))</f>
         <v>699</v>
       </c>
       <c r="G6" s="14">
@@ -1433,7 +1488,7 @@
         <v>0.46087912087912086</v>
       </c>
       <c r="J6" s="23">
-        <f>IFERROR(Tiers!$B$14*12/E6,0)</f>
+        <f>IFERROR(Tiers!$B$15*12/E6,0)</f>
         <v>0.46087912087912086</v>
       </c>
       <c r="K6" s="24">
@@ -1441,18 +1496,18 @@
         <v>0.9217582417582417</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B7" s="12">
         <v>30</v>
       </c>
       <c r="C7" s="19">
-        <f>B7*Tiers!$B$12</f>
+        <f>B7*Tiers!$B$13</f>
         <v>10920</v>
       </c>
       <c r="D7" s="20">
@@ -1463,7 +1518,7 @@
         <v>24024.000000000004</v>
       </c>
       <c r="F7" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(B7,Tiers!$B$5:$B$7,1))</f>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(B7,Tiers!$B$5:$B$8,1))</f>
         <v>699</v>
       </c>
       <c r="G7" s="14">
@@ -1479,7 +1534,7 @@
         <v>0.3491508491508491</v>
       </c>
       <c r="J7" s="23">
-        <f>IFERROR(Tiers!$B$14*12/E7,0)</f>
+        <f>IFERROR(Tiers!$B$15*12/E7,0)</f>
         <v>0.3491508491508491</v>
       </c>
       <c r="K7" s="24">
@@ -1492,13 +1547,13 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B8" s="12">
         <v>45</v>
       </c>
       <c r="C8" s="19">
-        <f>B8*Tiers!$B$12</f>
+        <f>B8*Tiers!$B$13</f>
         <v>16380</v>
       </c>
       <c r="D8" s="20">
@@ -1509,28 +1564,28 @@
         <v>39312</v>
       </c>
       <c r="F8" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(B8,Tiers!$B$5:$B$7,1))</f>
-        <v>1099</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(B8,Tiers!$B$5:$B$8,1))</f>
+        <v>999</v>
       </c>
       <c r="G8" s="14">
         <f>F8*12</f>
-        <v>13188</v>
+        <v>11988</v>
       </c>
       <c r="H8" s="14">
         <f>E8-G8</f>
-        <v>26124</v>
+        <v>27324</v>
       </c>
       <c r="I8" s="22">
         <f>IFERROR(G8/E8,0)</f>
-        <v>0.33547008547008544</v>
+        <v>0.30494505494505497</v>
       </c>
       <c r="J8" s="23">
-        <f>IFERROR(Tiers!$B$14*12/E8,0)</f>
+        <f>IFERROR(Tiers!$B$15*12/E8,0)</f>
         <v>0.21336996336996336</v>
       </c>
       <c r="K8" s="24">
         <f>IFERROR(G8/C8,0)</f>
-        <v>0.8051282051282052</v>
+        <v>0.7318681318681318</v>
       </c>
       <c r="L8" s="14">
         <v>116298</v>
@@ -1538,13 +1593,13 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B9" s="12">
         <v>55</v>
       </c>
       <c r="C9" s="19">
-        <f>B9*Tiers!$B$12</f>
+        <f>B9*Tiers!$B$13</f>
         <v>20020</v>
       </c>
       <c r="D9" s="20">
@@ -1555,28 +1610,28 @@
         <v>52052</v>
       </c>
       <c r="F9" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(B9,Tiers!$B$5:$B$7,1))</f>
-        <v>1099</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(B9,Tiers!$B$5:$B$8,1))</f>
+        <v>999</v>
       </c>
       <c r="G9" s="14">
         <f>F9*12</f>
-        <v>13188</v>
+        <v>11988</v>
       </c>
       <c r="H9" s="14">
         <f>E9-G9</f>
-        <v>38864</v>
+        <v>40064</v>
       </c>
       <c r="I9" s="22">
         <f>IFERROR(G9/E9,0)</f>
-        <v>0.25336202259279184</v>
+        <v>0.23030815338507646</v>
       </c>
       <c r="J9" s="23">
-        <f>IFERROR(Tiers!$B$14*12/E9,0)</f>
+        <f>IFERROR(Tiers!$B$15*12/E9,0)</f>
         <v>0.16114654576193038</v>
       </c>
       <c r="K9" s="24">
         <f>IFERROR(G9/C9,0)</f>
-        <v>0.6587412587412588</v>
+        <v>0.5988011988011988</v>
       </c>
       <c r="L9" s="14">
         <v>144144</v>
@@ -1584,13 +1639,13 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B10" s="12">
         <v>90</v>
       </c>
       <c r="C10" s="19">
-        <f>B10*Tiers!$B$12</f>
+        <f>B10*Tiers!$B$13</f>
         <v>32760</v>
       </c>
       <c r="D10" s="20">
@@ -1601,28 +1656,28 @@
         <v>75348</v>
       </c>
       <c r="F10" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(B10,Tiers!$B$5:$B$7,1))</f>
-        <v>1499</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(B10,Tiers!$B$5:$B$8,1))</f>
+        <v>1299</v>
       </c>
       <c r="G10" s="14">
         <f>F10*12</f>
-        <v>17988</v>
+        <v>15588</v>
       </c>
       <c r="H10" s="14">
         <f>E10-G10</f>
-        <v>57360</v>
+        <v>59760</v>
       </c>
       <c r="I10" s="22">
         <f>IFERROR(G10/E10,0)</f>
-        <v>0.23873228221054307</v>
+        <v>0.20688007644529383</v>
       </c>
       <c r="J10" s="23">
-        <f>IFERROR(Tiers!$B$14*12/E10,0)</f>
+        <f>IFERROR(Tiers!$B$15*12/E10,0)</f>
         <v>0.11132345914954611</v>
       </c>
       <c r="K10" s="24">
         <f>IFERROR(G10/C10,0)</f>
-        <v>0.5490842490842491</v>
+        <v>0.4758241758241758</v>
       </c>
       <c r="L10" s="14">
         <v>229320</v>
@@ -1630,13 +1685,13 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B11" s="12">
         <v>120</v>
       </c>
       <c r="C11" s="19">
-        <f>B11*Tiers!$B$12</f>
+        <f>B11*Tiers!$B$13</f>
         <v>43680</v>
       </c>
       <c r="D11" s="20">
@@ -1647,28 +1702,28 @@
         <v>100463.99999999999</v>
       </c>
       <c r="F11" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(B11,Tiers!$B$5:$B$7,1))</f>
-        <v>1499</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(B11,Tiers!$B$5:$B$8,1))</f>
+        <v>1599</v>
       </c>
       <c r="G11" s="14">
         <f>F11*12</f>
-        <v>17988</v>
+        <v>19188</v>
       </c>
       <c r="H11" s="14">
         <f>E11-G11</f>
-        <v>82475.99999999999</v>
+        <v>81275.99999999999</v>
       </c>
       <c r="I11" s="22">
         <f>IFERROR(G11/E11,0)</f>
-        <v>0.17904921165790733</v>
+        <v>0.1909937888198758</v>
       </c>
       <c r="J11" s="23">
-        <f>IFERROR(Tiers!$B$14*12/E11,0)</f>
+        <f>IFERROR(Tiers!$B$15*12/E11,0)</f>
         <v>0.0834925943621596</v>
       </c>
       <c r="K11" s="24">
         <f>IFERROR(G11/C11,0)</f>
-        <v>0.4118131868131868</v>
+        <v>0.4392857142857143</v>
       </c>
       <c r="L11" s="14">
         <v>305760</v>
@@ -1676,50 +1731,50 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E12" s="27">
         <f>SUM(E6:E11)</f>
         <v>309400</v>
       </c>
       <c r="F12" s="26" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="G12" s="27">
         <f>SUM(G6:G11)</f>
-        <v>79128</v>
+        <v>75528</v>
       </c>
       <c r="H12" s="27">
         <f>SUM(H6:H11)</f>
-        <v>230272</v>
+        <v>233872</v>
       </c>
       <c r="I12" s="28">
         <f>IFERROR(G12/E12,0)</f>
-        <v>0.25574660633484164</v>
+        <v>0.24411118293471235</v>
       </c>
       <c r="J12" s="29">
-        <f>IFERROR(Tiers!$B$14*12*6/E12,0)</f>
+        <f>IFERROR(Tiers!$B$15*12*6/E12,0)</f>
         <v>0.16266321913380738</v>
       </c>
       <c r="K12" s="26" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L12" s="26" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1743,13 +1798,13 @@
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1761,7 +1816,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1773,7 +1828,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B4" s="20">
         <v>2.3</v>
@@ -1781,31 +1836,31 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1813,7 +1868,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="19">
-        <f>A6*Tiers!$B$12</f>
+        <f>A6*Tiers!$B$13</f>
         <v>3640</v>
       </c>
       <c r="C6" s="14">
@@ -1821,7 +1876,7 @@
         <v>8372</v>
       </c>
       <c r="D6" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E6" s="30">
@@ -1829,7 +1884,7 @@
         <v>1.001911132345915</v>
       </c>
       <c r="F6" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A6,Tiers!$B$5:$B$7,1))*12</f>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A6,Tiers!$B$5:$B$8,1))*12</f>
         <v>8388</v>
       </c>
       <c r="G6" s="22">
@@ -1850,7 +1905,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="19">
-        <f>A7*Tiers!$B$12</f>
+        <f>A7*Tiers!$B$13</f>
         <v>5460</v>
       </c>
       <c r="C7" s="14">
@@ -1858,7 +1913,7 @@
         <v>12557.999999999998</v>
       </c>
       <c r="D7" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E7" s="30">
@@ -1866,7 +1921,7 @@
         <v>0.6679407548972768</v>
       </c>
       <c r="F7" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A7,Tiers!$B$5:$B$7,1))*12</f>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A7,Tiers!$B$5:$B$8,1))*12</f>
         <v>8388</v>
       </c>
       <c r="G7" s="22">
@@ -1887,7 +1942,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="19">
-        <f>A8*Tiers!$B$12</f>
+        <f>A8*Tiers!$B$13</f>
         <v>7280</v>
       </c>
       <c r="C8" s="14">
@@ -1895,7 +1950,7 @@
         <v>16744</v>
       </c>
       <c r="D8" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E8" s="30">
@@ -1903,7 +1958,7 @@
         <v>0.5009555661729574</v>
       </c>
       <c r="F8" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A8,Tiers!$B$5:$B$7,1))*12</f>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A8,Tiers!$B$5:$B$8,1))*12</f>
         <v>8388</v>
       </c>
       <c r="G8" s="22">
@@ -1924,7 +1979,7 @@
         <v>25</v>
       </c>
       <c r="B9" s="19">
-        <f>A9*Tiers!$B$12</f>
+        <f>A9*Tiers!$B$13</f>
         <v>9100</v>
       </c>
       <c r="C9" s="14">
@@ -1932,7 +1987,7 @@
         <v>20930</v>
       </c>
       <c r="D9" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E9" s="30">
@@ -1940,7 +1995,7 @@
         <v>0.400764452938366</v>
       </c>
       <c r="F9" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A9,Tiers!$B$5:$B$7,1))*12</f>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A9,Tiers!$B$5:$B$8,1))*12</f>
         <v>8388</v>
       </c>
       <c r="G9" s="22">
@@ -1961,7 +2016,7 @@
         <v>30</v>
       </c>
       <c r="B10" s="19">
-        <f>A10*Tiers!$B$12</f>
+        <f>A10*Tiers!$B$13</f>
         <v>10920</v>
       </c>
       <c r="C10" s="14">
@@ -1969,7 +2024,7 @@
         <v>25115.999999999996</v>
       </c>
       <c r="D10" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E10" s="30">
@@ -1977,7 +2032,7 @@
         <v>0.3339703774486384</v>
       </c>
       <c r="F10" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A10,Tiers!$B$5:$B$7,1))*12</f>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A10,Tiers!$B$5:$B$8,1))*12</f>
         <v>8388</v>
       </c>
       <c r="G10" s="22">
@@ -1998,7 +2053,7 @@
         <v>35</v>
       </c>
       <c r="B11" s="19">
-        <f>A11*Tiers!$B$12</f>
+        <f>A11*Tiers!$B$13</f>
         <v>12740</v>
       </c>
       <c r="C11" s="14">
@@ -2006,7 +2061,7 @@
         <v>29301.999999999996</v>
       </c>
       <c r="D11" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E11" s="30">
@@ -2014,7 +2069,7 @@
         <v>0.2862603235274043</v>
       </c>
       <c r="F11" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A11,Tiers!$B$5:$B$7,1))*12</f>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A11,Tiers!$B$5:$B$8,1))*12</f>
         <v>8388</v>
       </c>
       <c r="G11" s="22">
@@ -2035,7 +2090,7 @@
         <v>40</v>
       </c>
       <c r="B12" s="19">
-        <f>A12*Tiers!$B$12</f>
+        <f>A12*Tiers!$B$13</f>
         <v>14560</v>
       </c>
       <c r="C12" s="14">
@@ -2043,7 +2098,7 @@
         <v>33488</v>
       </c>
       <c r="D12" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E12" s="30">
@@ -2051,7 +2106,7 @@
         <v>0.2504777830864787</v>
       </c>
       <c r="F12" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A12,Tiers!$B$5:$B$7,1))*12</f>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A12,Tiers!$B$5:$B$8,1))*12</f>
         <v>8388</v>
       </c>
       <c r="G12" s="22">
@@ -2072,7 +2127,7 @@
         <v>45</v>
       </c>
       <c r="B13" s="19">
-        <f>A13*Tiers!$B$12</f>
+        <f>A13*Tiers!$B$13</f>
         <v>16380</v>
       </c>
       <c r="C13" s="14">
@@ -2080,7 +2135,7 @@
         <v>37674</v>
       </c>
       <c r="D13" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E13" s="30">
@@ -2088,20 +2143,20 @@
         <v>0.22264691829909222</v>
       </c>
       <c r="F13" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A13,Tiers!$B$5:$B$7,1))*12</f>
-        <v>13188</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A13,Tiers!$B$5:$B$8,1))*12</f>
+        <v>11988</v>
       </c>
       <c r="G13" s="22">
         <f>IFERROR(F13/C13,0)</f>
-        <v>0.3500557413600892</v>
+        <v>0.31820353559483994</v>
       </c>
       <c r="H13" s="14">
         <f>C13-F13</f>
-        <v>24486</v>
+        <v>25686</v>
       </c>
       <c r="I13" s="24">
         <f>IFERROR(F13/B13,0)</f>
-        <v>0.8051282051282052</v>
+        <v>0.7318681318681318</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -2109,7 +2164,7 @@
         <v>50</v>
       </c>
       <c r="B14" s="19">
-        <f>A14*Tiers!$B$12</f>
+        <f>A14*Tiers!$B$13</f>
         <v>18200</v>
       </c>
       <c r="C14" s="14">
@@ -2117,7 +2172,7 @@
         <v>41860</v>
       </c>
       <c r="D14" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E14" s="30">
@@ -2125,20 +2180,20 @@
         <v>0.200382226469183</v>
       </c>
       <c r="F14" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A14,Tiers!$B$5:$B$7,1))*12</f>
-        <v>13188</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A14,Tiers!$B$5:$B$8,1))*12</f>
+        <v>11988</v>
       </c>
       <c r="G14" s="22">
         <f>IFERROR(F14/C14,0)</f>
-        <v>0.31505016722408025</v>
+        <v>0.28638318203535595</v>
       </c>
       <c r="H14" s="14">
         <f>C14-F14</f>
-        <v>28672</v>
+        <v>29872</v>
       </c>
       <c r="I14" s="24">
         <f>IFERROR(F14/B14,0)</f>
-        <v>0.7246153846153847</v>
+        <v>0.6586813186813186</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -2146,7 +2201,7 @@
         <v>55</v>
       </c>
       <c r="B15" s="19">
-        <f>A15*Tiers!$B$12</f>
+        <f>A15*Tiers!$B$13</f>
         <v>20020</v>
       </c>
       <c r="C15" s="14">
@@ -2154,7 +2209,7 @@
         <v>46046</v>
       </c>
       <c r="D15" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E15" s="30">
@@ -2162,20 +2217,20 @@
         <v>0.18216566042652999</v>
       </c>
       <c r="F15" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A15,Tiers!$B$5:$B$7,1))*12</f>
-        <v>13188</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A15,Tiers!$B$5:$B$8,1))*12</f>
+        <v>11988</v>
       </c>
       <c r="G15" s="22">
         <f>IFERROR(F15/C15,0)</f>
-        <v>0.2864092429309821</v>
+        <v>0.26034834730486905</v>
       </c>
       <c r="H15" s="14">
         <f>C15-F15</f>
-        <v>32858</v>
+        <v>34058</v>
       </c>
       <c r="I15" s="24">
         <f>IFERROR(F15/B15,0)</f>
-        <v>0.6587412587412588</v>
+        <v>0.5988011988011988</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -2183,7 +2238,7 @@
         <v>60</v>
       </c>
       <c r="B16" s="19">
-        <f>A16*Tiers!$B$12</f>
+        <f>A16*Tiers!$B$13</f>
         <v>21840</v>
       </c>
       <c r="C16" s="14">
@@ -2191,7 +2246,7 @@
         <v>50231.99999999999</v>
       </c>
       <c r="D16" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E16" s="30">
@@ -2199,20 +2254,20 @@
         <v>0.1669851887243192</v>
       </c>
       <c r="F16" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A16,Tiers!$B$5:$B$7,1))*12</f>
-        <v>13188</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A16,Tiers!$B$5:$B$8,1))*12</f>
+        <v>11988</v>
       </c>
       <c r="G16" s="22">
         <f>IFERROR(F16/C16,0)</f>
-        <v>0.26254180602006694</v>
+        <v>0.23865265169612998</v>
       </c>
       <c r="H16" s="14">
         <f>C16-F16</f>
-        <v>37043.99999999999</v>
+        <v>38243.99999999999</v>
       </c>
       <c r="I16" s="24">
         <f>IFERROR(F16/B16,0)</f>
-        <v>0.6038461538461538</v>
+        <v>0.548901098901099</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -2220,7 +2275,7 @@
         <v>65</v>
       </c>
       <c r="B17" s="19">
-        <f>A17*Tiers!$B$12</f>
+        <f>A17*Tiers!$B$13</f>
         <v>23660</v>
       </c>
       <c r="C17" s="14">
@@ -2228,7 +2283,7 @@
         <v>54417.99999999999</v>
       </c>
       <c r="D17" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E17" s="30">
@@ -2236,20 +2291,20 @@
         <v>0.15414017420706386</v>
       </c>
       <c r="F17" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A17,Tiers!$B$5:$B$7,1))*12</f>
-        <v>13188</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A17,Tiers!$B$5:$B$8,1))*12</f>
+        <v>11988</v>
       </c>
       <c r="G17" s="22">
         <f>IFERROR(F17/C17,0)</f>
-        <v>0.24234628248006176</v>
+        <v>0.2202947554118123</v>
       </c>
       <c r="H17" s="14">
         <f>C17-F17</f>
-        <v>41229.99999999999</v>
+        <v>42429.99999999999</v>
       </c>
       <c r="I17" s="24">
         <f>IFERROR(F17/B17,0)</f>
-        <v>0.557396449704142</v>
+        <v>0.5066779374471683</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -2257,7 +2312,7 @@
         <v>70</v>
       </c>
       <c r="B18" s="19">
-        <f>A18*Tiers!$B$12</f>
+        <f>A18*Tiers!$B$13</f>
         <v>25480</v>
       </c>
       <c r="C18" s="14">
@@ -2265,7 +2320,7 @@
         <v>58603.99999999999</v>
       </c>
       <c r="D18" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E18" s="30">
@@ -2273,20 +2328,20 @@
         <v>0.14313016176370216</v>
       </c>
       <c r="F18" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A18,Tiers!$B$5:$B$7,1))*12</f>
-        <v>13188</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A18,Tiers!$B$5:$B$8,1))*12</f>
+        <v>11988</v>
       </c>
       <c r="G18" s="22">
         <f>IFERROR(F18/C18,0)</f>
-        <v>0.22503583373148595</v>
+        <v>0.20455941573953998</v>
       </c>
       <c r="H18" s="14">
         <f>C18-F18</f>
-        <v>45415.99999999999</v>
+        <v>46615.99999999999</v>
       </c>
       <c r="I18" s="24">
         <f>IFERROR(F18/B18,0)</f>
-        <v>0.5175824175824176</v>
+        <v>0.47048665620094193</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -2294,7 +2349,7 @@
         <v>75</v>
       </c>
       <c r="B19" s="19">
-        <f>A19*Tiers!$B$12</f>
+        <f>A19*Tiers!$B$13</f>
         <v>27300</v>
       </c>
       <c r="C19" s="14">
@@ -2302,7 +2357,7 @@
         <v>62789.99999999999</v>
       </c>
       <c r="D19" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E19" s="30">
@@ -2310,20 +2365,20 @@
         <v>0.13358815097945534</v>
       </c>
       <c r="F19" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A19,Tiers!$B$5:$B$7,1))*12</f>
-        <v>13188</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A19,Tiers!$B$5:$B$8,1))*12</f>
+        <v>15588</v>
       </c>
       <c r="G19" s="22">
         <f>IFERROR(F19/C19,0)</f>
-        <v>0.21003344481605354</v>
+        <v>0.24825609173435265</v>
       </c>
       <c r="H19" s="14">
         <f>C19-F19</f>
-        <v>49601.99999999999</v>
+        <v>47201.99999999999</v>
       </c>
       <c r="I19" s="24">
         <f>IFERROR(F19/B19,0)</f>
-        <v>0.48307692307692307</v>
+        <v>0.570989010989011</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -2331,7 +2386,7 @@
         <v>80</v>
       </c>
       <c r="B20" s="19">
-        <f>A20*Tiers!$B$12</f>
+        <f>A20*Tiers!$B$13</f>
         <v>29120</v>
       </c>
       <c r="C20" s="14">
@@ -2339,7 +2394,7 @@
         <v>66976</v>
       </c>
       <c r="D20" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E20" s="30">
@@ -2347,20 +2402,20 @@
         <v>0.12523889154323936</v>
       </c>
       <c r="F20" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A20,Tiers!$B$5:$B$7,1))*12</f>
-        <v>13188</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A20,Tiers!$B$5:$B$8,1))*12</f>
+        <v>15588</v>
       </c>
       <c r="G20" s="22">
         <f>IFERROR(F20/C20,0)</f>
-        <v>0.19690635451505017</v>
+        <v>0.23274008600095555</v>
       </c>
       <c r="H20" s="14">
         <f>C20-F20</f>
-        <v>53788</v>
+        <v>51388</v>
       </c>
       <c r="I20" s="24">
         <f>IFERROR(F20/B20,0)</f>
-        <v>0.4528846153846154</v>
+        <v>0.5353021978021978</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -2368,7 +2423,7 @@
         <v>85</v>
       </c>
       <c r="B21" s="19">
-        <f>A21*Tiers!$B$12</f>
+        <f>A21*Tiers!$B$13</f>
         <v>30940</v>
       </c>
       <c r="C21" s="14">
@@ -2376,7 +2431,7 @@
         <v>71162</v>
       </c>
       <c r="D21" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E21" s="30">
@@ -2384,20 +2439,20 @@
         <v>0.11787189792304882</v>
       </c>
       <c r="F21" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A21,Tiers!$B$5:$B$7,1))*12</f>
-        <v>17988</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A21,Tiers!$B$5:$B$8,1))*12</f>
+        <v>15588</v>
       </c>
       <c r="G21" s="22">
         <f>IFERROR(F21/C21,0)</f>
-        <v>0.25277535763469267</v>
+        <v>0.2190494927067817</v>
       </c>
       <c r="H21" s="14">
         <f>C21-F21</f>
-        <v>53174</v>
+        <v>55574</v>
       </c>
       <c r="I21" s="24">
         <f>IFERROR(F21/B21,0)</f>
-        <v>0.5813833225597932</v>
+        <v>0.5038138332255979</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -2405,7 +2460,7 @@
         <v>90</v>
       </c>
       <c r="B22" s="19">
-        <f>A22*Tiers!$B$12</f>
+        <f>A22*Tiers!$B$13</f>
         <v>32760</v>
       </c>
       <c r="C22" s="14">
@@ -2413,7 +2468,7 @@
         <v>75348</v>
       </c>
       <c r="D22" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E22" s="30">
@@ -2421,20 +2476,20 @@
         <v>0.11132345914954611</v>
       </c>
       <c r="F22" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A22,Tiers!$B$5:$B$7,1))*12</f>
-        <v>17988</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A22,Tiers!$B$5:$B$8,1))*12</f>
+        <v>15588</v>
       </c>
       <c r="G22" s="22">
         <f>IFERROR(F22/C22,0)</f>
-        <v>0.23873228221054307</v>
+        <v>0.20688007644529383</v>
       </c>
       <c r="H22" s="14">
         <f>C22-F22</f>
-        <v>57360</v>
+        <v>59760</v>
       </c>
       <c r="I22" s="24">
         <f>IFERROR(F22/B22,0)</f>
-        <v>0.5490842490842491</v>
+        <v>0.4758241758241758</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -2442,7 +2497,7 @@
         <v>95</v>
       </c>
       <c r="B23" s="19">
-        <f>A23*Tiers!$B$12</f>
+        <f>A23*Tiers!$B$13</f>
         <v>34580</v>
       </c>
       <c r="C23" s="14">
@@ -2450,7 +2505,7 @@
         <v>79534</v>
       </c>
       <c r="D23" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E23" s="30">
@@ -2458,20 +2513,20 @@
         <v>0.10546432972062263</v>
       </c>
       <c r="F23" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A23,Tiers!$B$5:$B$7,1))*12</f>
-        <v>17988</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A23,Tiers!$B$5:$B$8,1))*12</f>
+        <v>15588</v>
       </c>
       <c r="G23" s="22">
         <f>IFERROR(F23/C23,0)</f>
-        <v>0.22616742525209343</v>
+        <v>0.19599165136922575</v>
       </c>
       <c r="H23" s="14">
         <f>C23-F23</f>
-        <v>61546</v>
+        <v>63946</v>
       </c>
       <c r="I23" s="24">
         <f>IFERROR(F23/B23,0)</f>
-        <v>0.520185078079815</v>
+        <v>0.4507807981492192</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -2479,7 +2534,7 @@
         <v>100</v>
       </c>
       <c r="B24" s="19">
-        <f>A24*Tiers!$B$12</f>
+        <f>A24*Tiers!$B$13</f>
         <v>36400</v>
       </c>
       <c r="C24" s="14">
@@ -2487,7 +2542,7 @@
         <v>83720</v>
       </c>
       <c r="D24" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E24" s="30">
@@ -2495,20 +2550,20 @@
         <v>0.1001911132345915</v>
       </c>
       <c r="F24" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A24,Tiers!$B$5:$B$7,1))*12</f>
-        <v>17988</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A24,Tiers!$B$5:$B$8,1))*12</f>
+        <v>15588</v>
       </c>
       <c r="G24" s="22">
         <f>IFERROR(F24/C24,0)</f>
-        <v>0.21485905398948876</v>
+        <v>0.18619206880076444</v>
       </c>
       <c r="H24" s="14">
         <f>C24-F24</f>
-        <v>65732</v>
+        <v>68132</v>
       </c>
       <c r="I24" s="24">
         <f>IFERROR(F24/B24,0)</f>
-        <v>0.4941758241758242</v>
+        <v>0.42824175824175825</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -2516,7 +2571,7 @@
         <v>105</v>
       </c>
       <c r="B25" s="19">
-        <f>A25*Tiers!$B$12</f>
+        <f>A25*Tiers!$B$13</f>
         <v>38220</v>
       </c>
       <c r="C25" s="14">
@@ -2524,7 +2579,7 @@
         <v>87906</v>
       </c>
       <c r="D25" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E25" s="30">
@@ -2532,20 +2587,20 @@
         <v>0.09542010784246809</v>
       </c>
       <c r="F25" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A25,Tiers!$B$5:$B$7,1))*12</f>
-        <v>17988</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A25,Tiers!$B$5:$B$8,1))*12</f>
+        <v>19188</v>
       </c>
       <c r="G25" s="22">
         <f>IFERROR(F25/C25,0)</f>
-        <v>0.20462767046617977</v>
+        <v>0.21827861579414373</v>
       </c>
       <c r="H25" s="14">
         <f>C25-F25</f>
-        <v>69918</v>
+        <v>68718</v>
       </c>
       <c r="I25" s="24">
         <f>IFERROR(F25/B25,0)</f>
-        <v>0.4706436420722135</v>
+        <v>0.5020408163265306</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -2553,7 +2608,7 @@
         <v>110</v>
       </c>
       <c r="B26" s="19">
-        <f>A26*Tiers!$B$12</f>
+        <f>A26*Tiers!$B$13</f>
         <v>40040</v>
       </c>
       <c r="C26" s="14">
@@ -2561,7 +2616,7 @@
         <v>92092</v>
       </c>
       <c r="D26" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E26" s="30">
@@ -2569,20 +2624,20 @@
         <v>0.09108283021326499</v>
       </c>
       <c r="F26" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A26,Tiers!$B$5:$B$7,1))*12</f>
-        <v>17988</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A26,Tiers!$B$5:$B$8,1))*12</f>
+        <v>19188</v>
       </c>
       <c r="G26" s="22">
         <f>IFERROR(F26/C26,0)</f>
-        <v>0.19532641271771706</v>
+        <v>0.20835686053077357</v>
       </c>
       <c r="H26" s="14">
         <f>C26-F26</f>
-        <v>74104</v>
+        <v>72904</v>
       </c>
       <c r="I26" s="24">
         <f>IFERROR(F26/B26,0)</f>
-        <v>0.44925074925074926</v>
+        <v>0.4792207792207792</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -2590,7 +2645,7 @@
         <v>115</v>
       </c>
       <c r="B27" s="19">
-        <f>A27*Tiers!$B$12</f>
+        <f>A27*Tiers!$B$13</f>
         <v>41860</v>
       </c>
       <c r="C27" s="14">
@@ -2598,7 +2653,7 @@
         <v>96277.99999999999</v>
       </c>
       <c r="D27" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E27" s="30">
@@ -2606,20 +2661,20 @@
         <v>0.08712270716051436</v>
       </c>
       <c r="F27" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A27,Tiers!$B$5:$B$7,1))*12</f>
-        <v>17988</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A27,Tiers!$B$5:$B$8,1))*12</f>
+        <v>19188</v>
       </c>
       <c r="G27" s="22">
         <f>IFERROR(F27/C27,0)</f>
-        <v>0.18683395999085983</v>
+        <v>0.199297866594653</v>
       </c>
       <c r="H27" s="14">
         <f>C27-F27</f>
-        <v>78289.99999999999</v>
+        <v>77089.99999999999</v>
       </c>
       <c r="I27" s="24">
         <f>IFERROR(F27/B27,0)</f>
-        <v>0.4297181079789775</v>
+        <v>0.4583850931677019</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -2627,7 +2682,7 @@
         <v>120</v>
       </c>
       <c r="B28" s="19">
-        <f>A28*Tiers!$B$12</f>
+        <f>A28*Tiers!$B$13</f>
         <v>43680</v>
       </c>
       <c r="C28" s="14">
@@ -2635,7 +2690,7 @@
         <v>100463.99999999999</v>
       </c>
       <c r="D28" s="21">
-        <f>Tiers!$B$14*12</f>
+        <f>Tiers!$B$15*12</f>
         <v>8388</v>
       </c>
       <c r="E28" s="30">
@@ -2643,30 +2698,30 @@
         <v>0.0834925943621596</v>
       </c>
       <c r="F28" s="21">
-        <f>INDEX(Tiers!$D$5:$D$7,MATCH(A28,Tiers!$B$5:$B$7,1))*12</f>
-        <v>17988</v>
+        <f>INDEX(Tiers!$D$5:$D$8,MATCH(A28,Tiers!$B$5:$B$8,1))*12</f>
+        <v>19188</v>
       </c>
       <c r="G28" s="22">
         <f>IFERROR(F28/C28,0)</f>
-        <v>0.17904921165790733</v>
+        <v>0.1909937888198758</v>
       </c>
       <c r="H28" s="14">
         <f>C28-F28</f>
-        <v>82475.99999999999</v>
+        <v>81275.99999999999</v>
       </c>
       <c r="I28" s="24">
         <f>IFERROR(F28/B28,0)</f>
-        <v>0.4118131868131868</v>
+        <v>0.4392857142857143</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2681,7 +2736,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -2691,7 +2746,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2703,7 +2758,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2715,7 +2770,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B3" s="31"/>
       <c r="C3" s="31"/>
@@ -2724,132 +2779,132 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B6" s="13">
         <v>2200</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D6" s="24">
         <f>B6/($B$12*12)</f>
         <v>36.666666666666664</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B7" s="13">
         <v>3400</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D7" s="24">
         <f>B7/($B$12*12)</f>
         <v>56.666666666666664</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B8" s="13">
         <v>45</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D8" s="24">
         <f>B8</f>
         <v>45</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B9" s="13">
         <v>38</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D9" s="24">
         <f>B9</f>
         <v>38</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B10" s="13">
         <v>55</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D10" s="24">
         <f>B10</f>
         <v>55</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D11" s="33">
         <f>SUM(D6:D10)</f>
         <v>231.33333333333331</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B12" s="12">
         <v>5</v>
@@ -2857,24 +2912,24 @@
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B16" s="21">
         <f>Tiers!D5</f>
@@ -2895,11 +2950,11 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B17" s="21">
         <f>Tiers!D6</f>
-        <v>1099</v>
+        <v>999</v>
       </c>
       <c r="C17" s="24">
         <f>$D$11</f>
@@ -2907,20 +2962,20 @@
       </c>
       <c r="D17" s="24">
         <f>B17-C17</f>
-        <v>867.6666666666667</v>
+        <v>767.6666666666667</v>
       </c>
       <c r="E17" s="22">
         <f>IFERROR(D17/B17,0)</f>
-        <v>0.7895056111616622</v>
+        <v>0.7684351017684352</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B18" s="21">
         <f>Tiers!D7</f>
-        <v>1499</v>
+        <v>1299</v>
       </c>
       <c r="C18" s="24">
         <f>$D$11</f>
@@ -2928,16 +2983,37 @@
       </c>
       <c r="D18" s="24">
         <f>B18-C18</f>
-        <v>1267.6666666666667</v>
+        <v>1067.6666666666667</v>
       </c>
       <c r="E18" s="22">
         <f>IFERROR(D18/B18,0)</f>
-        <v>0.8456748943740272</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>118</v>
+        <v>0.8219142930459328</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="21">
+        <f>Tiers!D8</f>
+        <v>1599</v>
+      </c>
+      <c r="C19" s="24">
+        <f>$D$11</f>
+        <v>231.33333333333331</v>
+      </c>
+      <c r="D19" s="24">
+        <f>B19-C19</f>
+        <v>1367.6666666666667</v>
+      </c>
+      <c r="E19" s="22">
+        <f>IFERROR(D19/B19,0)</f>
+        <v>0.855326245570148</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2953,17 +3029,17 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="3" width="16" customWidth="1"/>
     <col min="4" max="7" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2975,7 +3051,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2987,30 +3063,30 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B6" s="12">
         <v>12</v>
@@ -3038,123 +3114,151 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B7" s="12">
         <v>6</v>
       </c>
       <c r="C7" s="21">
         <f>Tiers!D6</f>
-        <v>1099</v>
+        <v>999</v>
       </c>
       <c r="D7" s="14">
         <f>B7*C7</f>
-        <v>6594</v>
+        <v>5994</v>
       </c>
       <c r="E7" s="14">
         <f>D7*12</f>
-        <v>79128</v>
+        <v>71928</v>
       </c>
       <c r="F7" s="14">
         <f>B7*(C7-'Cost to serve'!$D$11)</f>
-        <v>5206</v>
+        <v>4606</v>
       </c>
       <c r="G7" s="14">
         <f>F7*12</f>
-        <v>62472</v>
+        <v>55272</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B8" s="12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" s="21">
         <f>Tiers!D7</f>
-        <v>1499</v>
+        <v>1299</v>
       </c>
       <c r="D8" s="14">
         <f>B8*C8</f>
-        <v>2998</v>
+        <v>3897</v>
       </c>
       <c r="E8" s="14">
         <f>D8*12</f>
-        <v>35976</v>
+        <v>46764</v>
       </c>
       <c r="F8" s="14">
         <f>B8*(C8-'Cost to serve'!$D$11)</f>
-        <v>2535.3333333333335</v>
+        <v>3203</v>
       </c>
       <c r="G8" s="14">
         <f>F8*12</f>
-        <v>30424</v>
+        <v>38436</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="B9" s="34">
-        <f>SUM(B6:B8)</f>
-        <v>20</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>78</v>
-      </c>
-      <c r="D9" s="27">
-        <f>SUM(D6:D8)</f>
-        <v>17980</v>
-      </c>
-      <c r="E9" s="27">
-        <f>SUM(E6:E8)</f>
-        <v>215760</v>
-      </c>
-      <c r="F9" s="27">
-        <f>SUM(F6:F8)</f>
-        <v>13353.333333333334</v>
-      </c>
-      <c r="G9" s="27">
-        <f>SUM(G6:G8)</f>
-        <v>160240</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="B12" s="14">
-        <f>B9*Tiers!$B$14*12</f>
-        <v>167760</v>
+      <c r="A9" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="12">
+        <v>1</v>
+      </c>
+      <c r="C9" s="21">
+        <f>Tiers!D8</f>
+        <v>1599</v>
+      </c>
+      <c r="D9" s="14">
+        <f>B9*C9</f>
+        <v>1599</v>
+      </c>
+      <c r="E9" s="14">
+        <f>D9*12</f>
+        <v>19188</v>
+      </c>
+      <c r="F9" s="14">
+        <f>B9*(C9-'Cost to serve'!$D$11)</f>
+        <v>1367.6666666666667</v>
+      </c>
+      <c r="G9" s="14">
+        <f>F9*12</f>
+        <v>16412</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="34">
+        <f>SUM(B6:B9)</f>
+        <v>22</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" s="27">
+        <f>SUM(D6:D9)</f>
+        <v>19878</v>
+      </c>
+      <c r="E10" s="27">
+        <f>D10*12</f>
+        <v>238536</v>
+      </c>
+      <c r="F10" s="27">
+        <f>SUM(F6:F9)</f>
+        <v>14788.666666666666</v>
+      </c>
+      <c r="G10" s="27">
+        <f>F10*12</f>
+        <v>177464</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="B13" s="35">
-        <f>E9</f>
-        <v>215760</v>
+      <c r="A13" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="B13" s="14">
+        <f>B10*Tiers!$B$15*12</f>
+        <v>184536</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="B14" s="36">
-        <f>B13-B12</f>
-        <v>48000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
+      </c>
+      <c r="B14" s="35">
+        <f>E10</f>
+        <v>238536</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="B15" s="36">
+        <f>B14-B13</f>
+        <v>54000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>